<commit_message>
filtrar dados da lista
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Warley Souza\Music\read_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EECD9FD5-FA40-4DC1-9C56-95360D3D6EE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8FBCCBA-41C7-4D73-A618-4CDA0950210B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,9 +39,6 @@
     <t>Date Tested</t>
   </si>
   <si>
-    <t xml:space="preserve">Density </t>
-  </si>
-  <si>
     <t>7 Day Result</t>
   </si>
   <si>
@@ -79,6 +76,9 @@
   </si>
   <si>
     <t>1G</t>
+  </si>
+  <si>
+    <t>Density</t>
   </si>
 </sst>
 </file>
@@ -568,7 +568,12 @@
   <cols>
     <col min="1" max="1" width="5.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.44140625" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -585,33 +590,33 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="7">
         <v>44449</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" s="7"/>
       <c r="E2" s="6"/>
@@ -623,13 +628,13 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" s="11">
         <v>44449</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" s="11"/>
       <c r="E3" s="13"/>
@@ -641,13 +646,13 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="17">
         <v>44449</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4" s="17"/>
       <c r="E4" s="16"/>
@@ -659,13 +664,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="11">
         <v>44449</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="10"/>
@@ -677,13 +682,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" s="17">
         <v>44449</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6" s="17"/>
       <c r="E6" s="16"/>
@@ -695,13 +700,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="11">
         <v>44449</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="11"/>
       <c r="E7" s="10"/>
@@ -713,13 +718,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="17">
         <v>44449</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" s="17"/>
       <c r="E8" s="16"/>

</xml_diff>